<commit_message>
feat: 添加 Guide/GuideStep Luban Schema 定义、Excel 配置表及生成产物
</commit_message>
<xml_diff>
--- a/Config/Excels/__enums__.xlsx
+++ b/Config/Excels/__enums__.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145">
   <si>
     <t>##var</t>
   </si>
@@ -413,6 +413,42 @@
   </si>
   <si>
     <t>特效</t>
+  </si>
+  <si>
+    <t>引导步骤类型</t>
+  </si>
+  <si>
+    <t>EStepType</t>
+  </si>
+  <si>
+    <t>无类型</t>
+  </si>
+  <si>
+    <t>ClickUI</t>
+  </si>
+  <si>
+    <t>点击UI</t>
+  </si>
+  <si>
+    <t>点击UI引导</t>
+  </si>
+  <si>
+    <t>Dialog</t>
+  </si>
+  <si>
+    <t>对话</t>
+  </si>
+  <si>
+    <t>对话引导</t>
+  </si>
+  <si>
+    <t>Wait</t>
+  </si>
+  <si>
+    <t>等待</t>
+  </si>
+  <si>
+    <t>等待步骤</t>
   </si>
 </sst>
 </file>
@@ -420,10 +456,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -449,7 +485,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="0"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -457,7 +493,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -473,35 +517,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -539,7 +554,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF9C0006"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -547,7 +562,29 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -569,9 +606,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -585,7 +621,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -630,13 +666,139 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -648,163 +810,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -859,9 +901,44 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -877,15 +954,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -908,8 +976,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -928,32 +996,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -962,10 +1004,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="9">
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
@@ -974,19 +1016,19 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
@@ -995,116 +1037,116 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="25" borderId="10">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="38" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="34" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="36" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="37" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="35" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1134,6 +1176,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -1191,11 +1236,6 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="00EE7228"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1462,7 +1502,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AK56"/>
+  <dimension ref="A1:AK60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="17.125" style="4" customWidth="1"/>
@@ -1503,10 +1543,10 @@
       <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="13"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:12">
       <c r="A2" s="5" t="s">
@@ -3266,6 +3306,99 @@
       <c r="K56" s="2"/>
       <c r="L56" s="2"/>
     </row>
+    <row r="57" spans="1:12">
+      <c r="A57" t="s">
+        <v>133</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C57" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D57" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="J57" s="11">
+        <v>0</v>
+      </c>
+      <c r="K57" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="L57" s="11"/>
+    </row>
+    <row r="58" spans="2:12">
+      <c r="B58" s="11"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="I58" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="J58" s="11">
+        <v>1</v>
+      </c>
+      <c r="K58" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="L58" s="11"/>
+    </row>
+    <row r="59" spans="2:12">
+      <c r="B59" s="11"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="J59" s="11">
+        <v>2</v>
+      </c>
+      <c r="K59" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="L59" s="11"/>
+    </row>
+    <row r="60" spans="2:12">
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="J60" s="11">
+        <v>3</v>
+      </c>
+      <c r="K60" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="L60" s="11"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="H1:L1"/>

</xml_diff>

<commit_message>
[AI]feat: 添加 Guide/GuideStep Luban Schema 定义、Excel 配置表及生成产物
</commit_message>
<xml_diff>
--- a/Config/Excels/__enums__.xlsx
+++ b/Config/Excels/__enums__.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145">
   <si>
     <t>##var</t>
   </si>
@@ -413,6 +413,42 @@
   </si>
   <si>
     <t>特效</t>
+  </si>
+  <si>
+    <t>引导步骤类型</t>
+  </si>
+  <si>
+    <t>EStepType</t>
+  </si>
+  <si>
+    <t>无类型</t>
+  </si>
+  <si>
+    <t>ClickUI</t>
+  </si>
+  <si>
+    <t>点击UI</t>
+  </si>
+  <si>
+    <t>点击UI引导</t>
+  </si>
+  <si>
+    <t>Dialog</t>
+  </si>
+  <si>
+    <t>对话</t>
+  </si>
+  <si>
+    <t>对话引导</t>
+  </si>
+  <si>
+    <t>Wait</t>
+  </si>
+  <si>
+    <t>等待</t>
+  </si>
+  <si>
+    <t>等待步骤</t>
   </si>
 </sst>
 </file>
@@ -420,10 +456,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
   <fonts count="21">
     <font>
@@ -449,7 +485,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="0"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -457,7 +493,15 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -473,35 +517,6 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="等线"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="等线"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -539,7 +554,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
+      <color rgb="FF9C0006"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -547,7 +562,29 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="等线"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="等线"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -569,9 +606,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF006100"/>
       <name val="等线"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -585,7 +621,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -630,13 +666,139 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -648,163 +810,43 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -859,9 +901,44 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -877,15 +954,6 @@
       </top>
       <bottom style="thin">
         <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -908,8 +976,8 @@
       <left/>
       <right/>
       <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -928,32 +996,6 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
@@ -962,10 +1004,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="22" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="9">
+    <xf numFmtId="0" fontId="2" fillId="28" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="25" borderId="11">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0">
@@ -974,19 +1016,19 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="12" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="16" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="24" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="3" fillId="32" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0">
@@ -995,116 +1037,116 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="7">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="27" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0">
+    <xf numFmtId="0" fontId="0" fillId="22" borderId="9">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="15" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="30" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="8">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="5">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="9">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="25" borderId="10">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="11" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="29" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="16" borderId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="12" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="21" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="8">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="20" borderId="11">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="5">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="36" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="35" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="3" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="13" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="27" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="34" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="31" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="30" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="38" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="26" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="33" borderId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="34" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="10" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="36" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="32" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="37" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="13" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="35" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="26" borderId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="28" borderId="0">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="24" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="23" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="37" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="29" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="18" borderId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1134,6 +1176,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1"/>
@@ -1191,11 +1236,6 @@
     <cellStyle name="60% - 强调文字颜色 6" xfId="48" builtinId="52"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <mruColors>
-      <color rgb="00EE7228"/>
-    </mruColors>
-  </colors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
@@ -1462,7 +1502,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AK56"/>
+  <dimension ref="A1:AK60"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="17.125" style="4" customWidth="1"/>
@@ -1503,10 +1543,10 @@
       <c r="H1" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="11"/>
-      <c r="J1" s="11"/>
-      <c r="K1" s="11"/>
-      <c r="L1" s="12"/>
+      <c r="I1" s="12"/>
+      <c r="J1" s="12"/>
+      <c r="K1" s="12"/>
+      <c r="L1" s="13"/>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:12">
       <c r="A2" s="5" t="s">
@@ -3266,6 +3306,99 @@
       <c r="K56" s="2"/>
       <c r="L56" s="2"/>
     </row>
+    <row r="57" spans="1:12">
+      <c r="A57" t="s">
+        <v>133</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>134</v>
+      </c>
+      <c r="C57" s="11" t="b">
+        <v>0</v>
+      </c>
+      <c r="D57" s="11" t="b">
+        <v>1</v>
+      </c>
+      <c r="E57" s="11"/>
+      <c r="F57" s="11"/>
+      <c r="G57" s="11"/>
+      <c r="H57" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="I57" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="J57" s="11">
+        <v>0</v>
+      </c>
+      <c r="K57" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="L57" s="11"/>
+    </row>
+    <row r="58" spans="2:12">
+      <c r="B58" s="11"/>
+      <c r="C58" s="11"/>
+      <c r="D58" s="11"/>
+      <c r="E58" s="11"/>
+      <c r="F58" s="11"/>
+      <c r="G58" s="11"/>
+      <c r="H58" s="11" t="s">
+        <v>136</v>
+      </c>
+      <c r="I58" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="J58" s="11">
+        <v>1</v>
+      </c>
+      <c r="K58" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="L58" s="11"/>
+    </row>
+    <row r="59" spans="2:12">
+      <c r="B59" s="11"/>
+      <c r="C59" s="11"/>
+      <c r="D59" s="11"/>
+      <c r="E59" s="11"/>
+      <c r="F59" s="11"/>
+      <c r="G59" s="11"/>
+      <c r="H59" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="I59" s="11" t="s">
+        <v>140</v>
+      </c>
+      <c r="J59" s="11">
+        <v>2</v>
+      </c>
+      <c r="K59" s="11" t="s">
+        <v>141</v>
+      </c>
+      <c r="L59" s="11"/>
+    </row>
+    <row r="60" spans="2:12">
+      <c r="B60" s="11"/>
+      <c r="C60" s="11"/>
+      <c r="D60" s="11"/>
+      <c r="E60" s="11"/>
+      <c r="F60" s="11"/>
+      <c r="G60" s="11"/>
+      <c r="H60" s="11" t="s">
+        <v>142</v>
+      </c>
+      <c r="I60" s="11" t="s">
+        <v>143</v>
+      </c>
+      <c r="J60" s="11">
+        <v>3</v>
+      </c>
+      <c r="K60" s="11" t="s">
+        <v>144</v>
+      </c>
+      <c r="L60" s="11"/>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="H1:L1"/>

</xml_diff>

<commit_message>
[AI]feat: 新增 UIConfig Luban Excel 配置表，Layer/TweenType 使用 EUILayer/EUITweenType 枚举
</commit_message>
<xml_diff>
--- a/Config/Excels/__enums__.xlsx
+++ b/Config/Excels/__enums__.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169">
   <si>
     <t>##var</t>
   </si>
@@ -449,6 +449,78 @@
   </si>
   <si>
     <t>等待步骤</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUILayer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WorldUI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">世界场景UI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MainUI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">主界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Normal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">一般全屏界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Window</t>
+  </si>
+  <si>
+    <t xml:space="preserve">窗口</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tips</t>
+  </si>
+  <si>
+    <t xml:space="preserve">提示</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Guide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">引导</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loading</t>
+  </si>
+  <si>
+    <t xml:space="preserve">加载界面</t>
+  </si>
+  <si>
+    <t xml:space="preserve">界面层级</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EUITweenType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">无动画</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">淡入淡出</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Custom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">自定义动画</t>
+  </si>
+  <si>
+    <t xml:space="preserve">动画类型</t>
   </si>
 </sst>
 </file>
@@ -1500,9 +1572,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr/>
-  <dimension ref="A1:AK60"/>
+  <dimension ref="A1:AK72"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="17.125" style="4" customWidth="1"/>
@@ -3399,6 +3471,198 @@
       </c>
       <c r="L60" s="11"/>
     </row>
+    <row r="61" s="2" customFormat="1" spans="1:12">
+      <c r="A61" s="2"/>
+      <c r="B61" s="2"/>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+      <c r="G61" s="2"/>
+      <c r="H61" s="2"/>
+      <c r="I61" s="2"/>
+      <c r="J61" s="2"/>
+      <c r="K61" s="2"/>
+      <c r="L61" s="2"/>
+    </row>
+    <row r="62" spans="1:12">
+      <c r="A62" t="s">
+        <v>11</v>
+      </c>
+      <c r="B62" t="s">
+        <v>145</v>
+      </c>
+      <c r="C62" t="b">
+        <v>0</v>
+      </c>
+      <c r="D62" t="b">
+        <v>1</v>
+      </c>
+      <c r="H62" t="s">
+        <v>146</v>
+      </c>
+      <c r="I62" t="s">
+        <v>147</v>
+      </c>
+      <c r="J62">
+        <v>0</v>
+      </c>
+      <c r="K62" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12">
+      <c r="H63" t="s">
+        <v>148</v>
+      </c>
+      <c r="I63" t="s">
+        <v>149</v>
+      </c>
+      <c r="J63">
+        <v>1500</v>
+      </c>
+      <c r="K63" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12">
+      <c r="H64" t="s">
+        <v>150</v>
+      </c>
+      <c r="I64" t="s">
+        <v>151</v>
+      </c>
+      <c r="J64">
+        <v>2000</v>
+      </c>
+      <c r="K64" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12">
+      <c r="H65" t="s">
+        <v>152</v>
+      </c>
+      <c r="I65" t="s">
+        <v>153</v>
+      </c>
+      <c r="J65">
+        <v>2500</v>
+      </c>
+      <c r="K65" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12">
+      <c r="H66" t="s">
+        <v>154</v>
+      </c>
+      <c r="I66" t="s">
+        <v>155</v>
+      </c>
+      <c r="J66">
+        <v>3000</v>
+      </c>
+      <c r="K66" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12">
+      <c r="H67" t="s">
+        <v>156</v>
+      </c>
+      <c r="I67" t="s">
+        <v>157</v>
+      </c>
+      <c r="J67">
+        <v>3500</v>
+      </c>
+      <c r="K67" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12">
+      <c r="H68" t="s">
+        <v>158</v>
+      </c>
+      <c r="I68" t="s">
+        <v>159</v>
+      </c>
+      <c r="J68">
+        <v>4000</v>
+      </c>
+      <c r="K68" t="s">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="69" s="2" customFormat="1" spans="1:12">
+      <c r="A69" s="2"/>
+      <c r="B69" s="2"/>
+      <c r="C69" s="2"/>
+      <c r="D69" s="2"/>
+      <c r="E69" s="2"/>
+      <c r="F69" s="2"/>
+      <c r="G69" s="2"/>
+      <c r="H69" s="2"/>
+      <c r="I69" s="2"/>
+      <c r="J69" s="2"/>
+      <c r="K69" s="2"/>
+      <c r="L69" s="2"/>
+    </row>
+    <row r="70" spans="1:12">
+      <c r="A70" t="s">
+        <v>11</v>
+      </c>
+      <c r="B70" t="s">
+        <v>161</v>
+      </c>
+      <c r="C70" t="b">
+        <v>0</v>
+      </c>
+      <c r="D70" t="b">
+        <v>1</v>
+      </c>
+      <c r="H70" t="s">
+        <v>162</v>
+      </c>
+      <c r="I70" t="s">
+        <v>163</v>
+      </c>
+      <c r="J70">
+        <v>0</v>
+      </c>
+      <c r="K70" t="s">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12">
+      <c r="H71" t="s">
+        <v>164</v>
+      </c>
+      <c r="I71" t="s">
+        <v>165</v>
+      </c>
+      <c r="J71">
+        <v>1</v>
+      </c>
+      <c r="K71" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12">
+      <c r="H72" t="s">
+        <v>166</v>
+      </c>
+      <c r="I72" t="s">
+        <v>167</v>
+      </c>
+      <c r="J72">
+        <v>2</v>
+      </c>
+      <c r="K72" t="s">
+        <v>167</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="H1:L1"/>

</xml_diff>